<commit_message>
Refactor split functionality: Implement split engine, excel reader/writer, and error handling
- Removed worker-exec.js as it is no longer needed.
- Added split/errors.js for custom error handling.
- Introduced split/excelReader.js and split/excelWriter.js for reading and writing Excel files.
- Created split/generate-split.js to handle the main split logic and validation.
- Implemented split/pathUtil.js for file path utilities.
- Added split/ruleManager.js to manage loading and saving rules.
- Developed split/splitEngine.js to execute the split logic based on defined rules.
- Created split/splitService.js to orchestrate the split task execution.
- Introduced split/splitTypes.js for type validation and normalization of sheet rules.
- Added split/styleCopier.js to handle copying styles and formatting between sheets.
</commit_message>
<xml_diff>
--- a/test/浙江华锐捷技术有限公司日报表.xlsx
+++ b/test/浙江华锐捷技术有限公司日报表.xlsx
@@ -2326,7 +2326,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="112">
+  <dxfs count="109">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3038,11 +3038,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
@@ -3069,16 +3064,6 @@
           <bgColor rgb="FFFF9900"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
     </dxf>
     <dxf>
       <fill>
@@ -38458,39 +38443,26 @@
   <conditionalFormatting sqref="D88:D89"/>
   <conditionalFormatting sqref="D93:D94"/>
   <conditionalFormatting sqref="D96:D97"/>
-  <conditionalFormatting sqref="H4:L85 H86:L90 H91:L91 H92:L92 H93:L94 H95:L98 H99:L99 H100:L100">
-    <cfRule type="cellIs" dxfId="101" priority="11" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="M4:M85 M86:M90 M91 M92 M93:M94 M95:M98 M99 M100">
-    <cfRule type="cellIs" dxfId="102" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="101" priority="13" operator="greaterThan">
       <formula>170</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="12" operator="lessThan">
+    <cfRule type="cellIs" dxfId="102" priority="12" operator="lessThan">
       <formula>100</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D101:D104 D105 D106:D108"/>
-  <conditionalFormatting sqref="H101:L104 H105:L105 H106:L108">
-    <cfRule type="cellIs" dxfId="106" priority="7" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="3" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="M101:M104 M105 M106:M108">
-    <cfRule type="cellIs" dxfId="108" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="105" priority="9" operator="greaterThan">
       <formula>170</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="8" operator="lessThan">
+    <cfRule type="cellIs" dxfId="106" priority="8" operator="lessThan">
       <formula>100</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="107" priority="5" operator="greaterThan">
       <formula>170</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="108" priority="4" operator="lessThan">
       <formula>100</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>